<commit_message>
fix(carga): separa Ejecutivo Comercial del Asesor Pedagógico
El «Ejecutivo Responsable» del archivo de BI es la figura COMERCIAL: ahora se
guarda solo como dato del colegio (análisis/filtros) y nunca se convierte en
asesor. La columna nueva «Asesor Pedagógico» es quien se casa con un asesor
existente (o se crea) y recibe el colegio asignado.

- Plantilla: columna «Asesor Pedagógico» tras el ejecutivo; instrucciones y
  ejemplos distinguen ambas figuras (regenerada).
- Parser: alias separados («asesor» ya no mapea a ejecutivo); FilaColegio.asesorPed.
- Rentabilidad: agrupación nueva «Por ejecutivo» (comercial) junto a la de asesor.
- Prueba anti-confusión: el ejecutivo solo no crea asesor ni asigna, pero sí se
  guarda como dato (79 pruebas en total).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-colegios.xlsx
+++ b/public/plantilla-colegios.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:S4"/>
   <cols>
     <col min="1" max="1" width="19.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -408,16 +408,17 @@
     <col min="6" max="6" width="23.83203125" customWidth="1"/>
     <col min="7" max="7" width="22.83203125" customWidth="1"/>
     <col min="8" max="8" width="23.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" customWidth="1"/>
-    <col min="15" max="15" width="17.83203125" customWidth="1"/>
-    <col min="16" max="16" width="19.83203125" customWidth="1"/>
-    <col min="17" max="17" width="21.83203125" customWidth="1"/>
-    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="19.83203125" customWidth="1"/>
+    <col min="16" max="16" width="17.83203125" customWidth="1"/>
+    <col min="17" max="17" width="19.83203125" customWidth="1"/>
+    <col min="18" max="18" width="21.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,33 +447,36 @@
         <v>Ejecutivo Responsable</v>
       </c>
       <c r="I1" t="str">
+        <v>Asesor Pedagógico</v>
+      </c>
+      <c r="J1" t="str">
         <v>Años de Antigüedad</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Serie Preescolar</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Serie Primaria</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Serie Secundaria</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Bachillerato</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Inglés Preescolar</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Inglés Primaria</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Inglés Secundaria</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Inglés Bachillerato</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Otra Serie</v>
       </c>
     </row>
@@ -501,11 +505,11 @@
       <c r="H2" t="str">
         <v>Mariana López</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="str">
+        <v>Laura Sánchez</v>
+      </c>
+      <c r="J2">
         <v>12</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Acierta</v>
       </c>
       <c r="K2" t="str">
         <v>Acierta</v>
@@ -514,21 +518,24 @@
         <v>Acierta</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>Acierta</v>
       </c>
       <c r="N2" t="str">
-        <v>Bright Sparks</v>
+        <v/>
       </c>
       <c r="O2" t="str">
         <v>Bright Sparks</v>
       </c>
       <c r="P2" t="str">
+        <v>Bright Sparks</v>
+      </c>
+      <c r="Q2" t="str">
         <v>Winglish</v>
       </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
       <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
         <v/>
       </c>
     </row>
@@ -557,34 +564,37 @@
       <c r="H3" t="str">
         <v>Jorge Ramírez</v>
       </c>
-      <c r="I3">
+      <c r="I3" t="str">
+        <v>Pedro Gómez</v>
+      </c>
+      <c r="J3">
         <v>5</v>
       </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
       <c r="K3" t="str">
-        <v>Revuela Up</v>
+        <v/>
       </c>
       <c r="L3" t="str">
         <v>Revuela Up</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>Revuela Up</v>
       </c>
       <c r="N3" t="str">
         <v/>
       </c>
       <c r="O3" t="str">
-        <v>Winglish</v>
+        <v/>
       </c>
       <c r="P3" t="str">
         <v>Winglish</v>
       </c>
       <c r="Q3" t="str">
-        <v/>
+        <v>Winglish</v>
       </c>
       <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
         <v/>
       </c>
     </row>
@@ -613,18 +623,18 @@
       <c r="H4" t="str">
         <v>Jorge Ramírez</v>
       </c>
-      <c r="I4">
+      <c r="I4" t="str">
+        <v>Pedro Gómez</v>
+      </c>
+      <c r="J4">
         <v>22</v>
       </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
       <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
         <v>Revuela Up</v>
       </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
       <c r="M4" t="str">
         <v/>
       </c>
@@ -641,19 +651,22 @@
         <v/>
       </c>
       <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
         <v>Serie legada 2019</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -784,40 +797,40 @@
         <v>Texto (nombre completo)</v>
       </c>
       <c r="D9" t="str">
-        <v>Se convierte en el asesor del colegio: si no existe se crea y el colegio queda asignado a él.</v>
+        <v>Ejecutivo COMERCIAL responsable del colegio. Queda como dato para análisis y filtros; NO es el asesor pedagógico y no asigna servicios.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Años de Antigüedad</v>
+        <v>Asesor Pedagógico</v>
       </c>
       <c r="B10" t="str">
-        <v>No</v>
+        <v>Recomendada</v>
       </c>
       <c r="C10" t="str">
-        <v>Número</v>
+        <v>Texto (nombre completo)</v>
       </c>
       <c r="D10" t="str">
-        <v>Años como cliente de SM.</v>
+        <v>Asesor que atiende los servicios académicos. Se convierte en el asesor del colegio: si no existe se crea y el colegio queda asignado a él.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Serie Preescolar</v>
+        <v>Años de Antigüedad</v>
       </c>
       <c r="B11" t="str">
         <v>No</v>
       </c>
       <c r="C11" t="str">
-        <v>Texto</v>
+        <v>Número</v>
       </c>
       <c r="D11" t="str">
-        <v>Serie que usa en ese nivel (vacío = no aplica).</v>
+        <v>Años como cliente de SM.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Serie Primaria</v>
+        <v>Serie Preescolar</v>
       </c>
       <c r="B12" t="str">
         <v>No</v>
@@ -826,12 +839,12 @@
         <v>Texto</v>
       </c>
       <c r="D12" t="str">
-        <v/>
+        <v>Serie que usa en ese nivel (vacío = no aplica).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Serie Secundaria</v>
+        <v>Serie Primaria</v>
       </c>
       <c r="B13" t="str">
         <v>No</v>
@@ -845,7 +858,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Bachillerato</v>
+        <v>Serie Secundaria</v>
       </c>
       <c r="B14" t="str">
         <v>No</v>
@@ -854,12 +867,12 @@
         <v>Texto</v>
       </c>
       <c r="D14" t="str">
-        <v>Serie de bachillerato (vacío = no aplica).</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Inglés Preescolar</v>
+        <v>Bachillerato</v>
       </c>
       <c r="B15" t="str">
         <v>No</v>
@@ -868,12 +881,12 @@
         <v>Texto</v>
       </c>
       <c r="D15" t="str">
-        <v>Programa de inglés en ese nivel.</v>
+        <v>Serie de bachillerato (vacío = no aplica).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Inglés Primaria</v>
+        <v>Inglés Preescolar</v>
       </c>
       <c r="B16" t="str">
         <v>No</v>
@@ -882,12 +895,12 @@
         <v>Texto</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>Programa de inglés en ese nivel.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Inglés Secundaria</v>
+        <v>Inglés Primaria</v>
       </c>
       <c r="B17" t="str">
         <v>No</v>
@@ -901,7 +914,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Inglés Bachillerato</v>
+        <v>Inglés Secundaria</v>
       </c>
       <c r="B18" t="str">
         <v>No</v>
@@ -915,49 +928,63 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>Inglés Bachillerato</v>
+      </c>
+      <c r="B19" t="str">
+        <v>No</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
         <v>Otra Serie</v>
       </c>
-      <c r="B19" t="str">
-        <v>No</v>
-      </c>
-      <c r="C19" t="str">
-        <v>Texto</v>
-      </c>
-      <c r="D19" t="str">
+      <c r="B20" t="str">
+        <v>No</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D20" t="str">
         <v>Cualquier otra serie no contemplada arriba.</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Formato</v>
-      </c>
-      <c r="B21" t="str">
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <v/>
-      </c>
-      <c r="D21" t="str">
-        <v>Una fila por colegio. No cambiar los encabezados. Se acepta .xlsx o .csv (UTF-8).</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>Formato</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v>Una fila por colegio. No cambiar los encabezados. Se acepta .xlsx o .csv (UTF-8).</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
         <v>Ejemplos</v>
       </c>
-      <c r="B22" t="str">
-        <v/>
-      </c>
-      <c r="C22" t="str">
-        <v/>
-      </c>
-      <c r="D22" t="str">
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v/>
+      </c>
+      <c r="D23" t="str">
         <v>Las 3 filas de la hoja «Colegios» son de ejemplo: bórrenlas antes de entregar.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>